<commit_message>
Added summarization key as Excel.
</commit_message>
<xml_diff>
--- a/p_gps_pts.xlsx
+++ b/p_gps_pts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{482DCFCD-CB29-4C6F-A4E2-D15E2062173E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C04B233-E9A2-4D28-9E31-7FF6BE17617E}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{482DCFCD-CB29-4C6F-A4E2-D15E2062173E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08A187CE-FE0C-4EAD-A94B-5CA8F6636FC5}"/>
   <bookViews>
     <workbookView xWindow="90" yWindow="45" windowWidth="28320" windowHeight="15330" xr2:uid="{472C6C18-3318-42E5-B3DE-BCE9F97FEFF7}"/>
   </bookViews>
@@ -3044,8 +3044,8 @@
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="17.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Add Excel version of summaries.
</commit_message>
<xml_diff>
--- a/p_gps_pts.xlsx
+++ b/p_gps_pts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{482DCFCD-CB29-4C6F-A4E2-D15E2062173E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08A187CE-FE0C-4EAD-A94B-5CA8F6636FC5}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{482DCFCD-CB29-4C6F-A4E2-D15E2062173E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8C550D9-258D-407C-BB9C-DC781A5739B4}"/>
   <bookViews>
     <workbookView xWindow="90" yWindow="45" windowWidth="28320" windowHeight="15330" xr2:uid="{472C6C18-3318-42E5-B3DE-BCE9F97FEFF7}"/>
   </bookViews>
@@ -3052,8 +3052,8 @@
     <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="22.7109375" bestFit="1" customWidth="1"/>

</xml_diff>